<commit_message>
Feat(Route_Optimiser): updated route algorythm logic, and improve UI
</commit_message>
<xml_diff>
--- a/BlueSG/rider_roster.xlsx
+++ b/BlueSG/rider_roster.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HRteam\Desktop\Lance\BlueSG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42403C66-905C-4248-B940-ABD7C65E66C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75646E9B-0AE1-478C-9C0F-C4B2C84A03F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monday" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="31">
   <si>
     <t>Rider Name</t>
   </si>
@@ -83,19 +83,61 @@
   </si>
   <si>
     <t>Central</t>
+  </si>
+  <si>
+    <t>Bedok</t>
+  </si>
+  <si>
+    <t>Abdul Rashid Bin Abdul Majid</t>
+  </si>
+  <si>
+    <t>Woodlands</t>
+  </si>
+  <si>
+    <t>Sadiq Batcha Mohamed Yusoof Mahadir</t>
+  </si>
+  <si>
+    <t>Syed Muhammad Faiq Bin Bagal</t>
+  </si>
+  <si>
+    <t>Lim Choon Yong Lester</t>
+  </si>
+  <si>
+    <t>Mohamed Sadhik Mohamed Yusof</t>
+  </si>
+  <si>
+    <t>Chen Yen Zong (El-Tian)</t>
+  </si>
+  <si>
+    <t>Fareed</t>
+  </si>
+  <si>
+    <t>Boon Keng</t>
+  </si>
+  <si>
+    <t>Whampoa</t>
+  </si>
+  <si>
+    <t>Toa Payoh</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -106,7 +148,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -114,12 +156,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -610,76 +671,125 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2">
+      <c r="A2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3">
+      <c r="A3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5">
+      <c r="D5" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="4">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement core project structure including vehicle route optimizer, conversion utilities, and tracker modules
</commit_message>
<xml_diff>
--- a/BlueSG/rider_roster.xlsx
+++ b/BlueSG/rider_roster.xlsx
@@ -1299,7 +1299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1327,37 +1327,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rider A</t>
+          <t>Lon</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sengkang</t>
+          <t>Marsiling</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rider B</t>
+          <t>Abdul Rashid Bin Abdul Majid</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Balestier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1367,12 +1367,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rider C</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1381,27 +1381,107 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rider D</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tampines</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Aaron Singh</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sembawang</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Safuwan</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Woodlands</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Chong Zhen Yang (Michael)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Compassvale</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>North-East</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mohammad Fareed Bin Mohammad Rashid</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Queenstown</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1415,7 +1495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1443,52 +1523,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rider A</t>
+          <t>Lon</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sengkang</t>
+          <t>Marsiling</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rider B</t>
+          <t>Ryan Oh</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Tampaines</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rider C</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1497,27 +1577,127 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rider D</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tampines</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sadiq Batcha Mohamed Yusoof Mahadir</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Toa Payoh</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Aaron Singh</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sembawang</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Safuwan</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Woodlands</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tee Boon Chuan (Jayson )</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Woodlands</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Zhi Ming</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tampaines</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>East</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>5</v>
+      <c r="D10" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>